<commit_message>
Correction retour à la ligne ffaeac2d5c0fa7ed987202ddb2cfdf7a02a6466d
</commit_message>
<xml_diff>
--- a/ressourcesCDA/ig/StructureDefinition-fr-cda-informant.xlsx
+++ b/ressourcesCDA/ig/StructureDefinition-fr-cda-informant.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-25T10:04:45+00:00</t>
+    <t>2026-02-26T08:51:17+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -431,11 +431,11 @@
 </t>
   </si>
   <si>
-    <t>**Informateur non professionnel** ayant fourni des informations relatives au document.
-- Ou : Personne de confiance désignée par le patient/usager.
-- Ou : Personne à prévenir en cas d’urgence.
-- Ou : Aidant du patient/usager.
-- Ou : Personne aidée</t>
+    <t>Informateur non professionnel ayant fourni des informations relatives au document.
+  Ou : Personne de confiance désignée par le patient/usager.
+  Ou : Personne à prévenir en cas d’urgence.
+  Ou : Aidant du patient/usager.
+  Ou : Personne aidée</t>
   </si>
 </sst>
 </file>
@@ -2236,10 +2236,10 @@
       <c r="K15" t="s" s="2">
         <v>134</v>
       </c>
-      <c r="L15" s="2"/>
-      <c r="M15" t="s" s="2">
+      <c r="L15" t="s" s="2">
         <v>135</v>
       </c>
+      <c r="M15" s="2"/>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
       <c r="P15" t="s" s="2">

</xml_diff>